<commit_message>
WIP: stage-3 fix round in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWExrN7wNZ4prKGqMsXc4Z
</commit_message>
<xml_diff>
--- a/public/downloads/schedule-template.xlsx
+++ b/public/downloads/schedule-template.xlsx
@@ -624,7 +624,7 @@
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>כתבו כאן נוסחה (צעד 1)</t>
+          <t>את הנוסחה כותבים בתא B10 (צעד 1), לא בתא הזה</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>כתבו כאן נוסחה (צעד 2)</t>
+          <t>את הנוסחה כותבים בתא B11 (צעד 2), לא בתא הזה</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: stage-3 final fixes and stage-1/2 videos in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWExrN7wNZ4prKGqMsXc4Z
</commit_message>
<xml_diff>
--- a/public/downloads/schedule-template.xlsx
+++ b/public/downloads/schedule-template.xlsx
@@ -654,7 +654,7 @@
           <t>ההחזר בחודש האחרון</t>
         </is>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="10" t="str">
         <f>IF(COUNT(C20:C379)=0,"",INDEX(C20:C379,B7))</f>
         <v/>
       </c>
@@ -667,7 +667,7 @@
       </c>
       <c r="B14" s="10">
         <f>SUM(C20:C379)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -678,7 +678,7 @@
       </c>
       <c r="B15" s="10">
         <f>SUM(D20:D379)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -689,7 +689,7 @@
       </c>
       <c r="B16" s="10">
         <f>SUM(E20:E379)</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
@@ -698,9 +698,9 @@
           <t>בדיקה</t>
         </is>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="11" t="str">
         <f>IF(COUNT(F20:F379)=0,"עוד לא מילאתם את הלוח",IF(AND(ABS(B16-B5)&lt;0.005,ABS(INDEX(F20:F379,B7))&lt;0.005),"✓ הלוח סוגר: הקרן שהוחזרה שווה להלוואה, והיתרה בסוף היא 0","✗ הלוח לא סוגר. בדקו את הנוסחאות, ושהעתקתם בדיוק עד החודש האחרון"))</f>
-        <v/>
+        <v>עוד לא מילאתם את הלוח</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">

</xml_diff>